<commit_message>
Fix: a bill never makes a second copy of a customer or supplier (Epic 11 Sprint 4 NF-4.26)
Found validating Epic 11 Sprint 12: a bill's own party list still matched on
the exact name only (only invoice lines asked the shared matcher), so a bill
from "Toyota Kirloskar Pvt. Ltd." made a second Toyota beside "Toyota
Kirloskar Pvt Ltd". Both paths now ask services/parties, read once per import
and kept current as the bill adds records. A Needs-details record takes the
bill's phone, email and address (blank fields only) and a phone ends its Needs
details, as the code's comment promised.

Tests: three new in test_everything_links_to_crm.py (bill finds the firm on
the other side and fills the GSTIN, Needs-details record completed by the
bill; a reused task takes the decision's party and keeps its own; renaming a
firm renames it on tasks and meetings). CRM suites 35 passed; full suite green
apart from the two known flakes (pass alone).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Master_Tracker.xlsx
+++ b/docs/DecisionOS_Master_Tracker.xlsx
@@ -585,7 +585,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>All-epics progress: 1060 of 1185 items resolved  (89%)</t>
+          <t>All-epics progress: 1065 of 1190 items resolved  (89%)</t>
         </is>
       </c>
     </row>
@@ -968,10 +968,10 @@
         </is>
       </c>
       <c r="C16" s="9" t="n">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>

</xml_diff>